<commit_message>
feat(solver): add soft constraints, asymmetric penalties, and global quarterly balancing
Stage2 MIP solver improvements:
- Asymmetric quarterly penalties (overshoot=100, undershoot=10)
- Global quarterly overshoot/undershoot penalty (500/5)
- Special rule annual/period constraints as soft (penalty=500)
- im-Durchlauf protection (can_stop=0) in bootstrap
- Large order penalty and existing small amount penalty
- OPT-row dedup fix in report_massnahmenplan

Config: SolverConfig extended with soft_target_undershoot_penalty,
global_quarter_overshoot_penalty, global_quarter_undershoot_penalty,
special_rule_annual_penalty. Tests updated accordingly.
</commit_message>
<xml_diff>
--- a/userdata/budget/planning/budget_sondervereinbarungen_ekek1.xlsx
+++ b/userdata/budget/planning/budget_sondervereinbarungen_ekek1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="16638" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20060" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="10">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -28,126 +28,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF9C5700"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color theme="0"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -205,201 +85,21 @@
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFF0000"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -407,209 +107,61 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.3999755851924192"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="48">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="45">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="45">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -631,55 +183,14 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="48">
+  <cellStyles count="7">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift" xfId="1" builtinId="15"/>
-    <cellStyle name="Überschrift 1" xfId="2" builtinId="16"/>
-    <cellStyle name="Überschrift 2" xfId="3" builtinId="17"/>
-    <cellStyle name="Überschrift 3" xfId="4" builtinId="18"/>
-    <cellStyle name="Überschrift 4" xfId="5" builtinId="19"/>
-    <cellStyle name="Gut" xfId="6" builtinId="26"/>
-    <cellStyle name="Schlecht" xfId="7" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28"/>
-    <cellStyle name="Eingabe" xfId="9" builtinId="20"/>
-    <cellStyle name="Ausgabe" xfId="10" builtinId="21"/>
-    <cellStyle name="Berechnung" xfId="11" builtinId="22"/>
-    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24"/>
-    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23"/>
-    <cellStyle name="Warnender Text" xfId="14" builtinId="11"/>
-    <cellStyle name="Notiz" xfId="15" builtinId="10"/>
-    <cellStyle name="Erklärender Text" xfId="16" builtinId="53"/>
-    <cellStyle name="Ergebnis" xfId="17" builtinId="25"/>
-    <cellStyle name="Akzent1" xfId="18" builtinId="29"/>
-    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30"/>
-    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31"/>
-    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32"/>
-    <cellStyle name="Akzent2" xfId="22" builtinId="33"/>
-    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34"/>
-    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35"/>
-    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36"/>
-    <cellStyle name="Akzent3" xfId="26" builtinId="37"/>
-    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38"/>
-    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39"/>
-    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40"/>
-    <cellStyle name="Akzent4" xfId="30" builtinId="41"/>
-    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42"/>
-    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43"/>
-    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44"/>
-    <cellStyle name="Akzent5" xfId="34" builtinId="45"/>
-    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46"/>
-    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47"/>
-    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48"/>
-    <cellStyle name="Akzent6" xfId="38" builtinId="49"/>
-    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50"/>
-    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51"/>
-    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52"/>
-    <cellStyle name="Standard 2" xfId="42"/>
-    <cellStyle name="Komma 2" xfId="43"/>
-    <cellStyle name="Währung 2" xfId="44"/>
-    <cellStyle name="Hyperlink" xfId="45"/>
-    <cellStyle name="Standard 3" xfId="46"/>
-    <cellStyle name="Komma 4" xfId="47"/>
+    <cellStyle name="Standard 2" xfId="1"/>
+    <cellStyle name="Komma 2" xfId="2"/>
+    <cellStyle name="Währung 2" xfId="3"/>
+    <cellStyle name="Hyperlink" xfId="4"/>
+    <cellStyle name="Standard 3" xfId="5"/>
+    <cellStyle name="Komma 4" xfId="6"/>
   </cellStyles>
   <dxfs count="7">
     <dxf>
@@ -1213,7 +724,8 @@
     <col width="48.140625" customWidth="1" style="10" min="5" max="5"/>
     <col width="11.42578125" customWidth="1" style="10" min="6" max="6"/>
     <col width="81.42578125" customWidth="1" style="10" min="7" max="7"/>
-    <col width="11.42578125" customWidth="1" style="10" min="8" max="16384"/>
+    <col width="11.42578125" customWidth="1" style="10" min="8" max="8"/>
+    <col width="11.42578125" customWidth="1" style="10" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.55" customHeight="1">
@@ -1486,7 +998,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42.8" customHeight="1">
+    <row r="11" ht="54.2" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
           <t>BIB+China Audi</t>
@@ -1513,8 +1025,8 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>EL und FL müssen exakt passen!
-Nur für EDAG!</t>
+          <t>folgende firmen buchen: EDAG
+Zur Not auch andere Firmen/Dienstleister, die woanders abgelehnt werden (prio 2). EA-Target bleibt unverändert.</t>
         </is>
       </c>
     </row>
@@ -1549,8 +1061,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="8" verticalDpi="0"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000d_</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000d_&amp;"Aptos Narrow"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000d_</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>

</xml_diff>